<commit_message>
Website: new base rate list (24 Oct 2026), drop items not on it, photos by item code
- Website Rates xlsx: 38 base rates updated from RCRT MIX UPDATED (old rate
  kept in the Note column); the 6 catalogue items with no rate (RC 200, 968,
  959, RC 307, RC 271, RC 262) removed.
- Catalogue: pages of those items left out; the 968/965 page is now 965.
  Unused images are cleaned out of public/img.
- Build: item photos from website/photos/ or website/New items*/, file name =
  item code ("D-01.jpg", "RC-610 (2).jpg"); added to the item's existing
  card or as a new card. Unmatched file names are listed.
- Site: a rate links to a photo by its own code when the sheet's
  "Catalogue item" column is empty.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XttcUphWVwshiXCPpeS9yb
</commit_message>
<xml_diff>
--- a/website/Website Rates (for Google Sheet).xlsx
+++ b/website/Website Rates (for Google Sheet).xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H146"/>
+  <dimension ref="A1:H140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -721,7 +721,6 @@
           <t>T-100</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -733,7 +732,6 @@
       <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>Y</t>
@@ -751,7 +749,6 @@
           <t>TESLA-701</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -781,14 +778,13 @@
           <t>TESLA-702</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Clutchers</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>60</v>
+        <v>108</v>
       </c>
       <c r="E10" t="n">
         <v>6</v>
@@ -803,7 +799,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr"/>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹60 → ₹108.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -811,7 +811,6 @@
           <t>TESLA-703</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -841,7 +840,6 @@
           <t>TESLA-707</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -871,7 +869,6 @@
           <t>TESLA-710</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -901,7 +898,6 @@
           <t>TESLA-711</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -931,7 +927,6 @@
           <t>TESLA-712</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -961,7 +956,6 @@
           <t>TESLA-713</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -991,7 +985,6 @@
           <t>TESLA-714</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1055,7 +1048,6 @@
           <t>TESLA-716</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1085,7 +1077,6 @@
           <t>TESLA-717</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1115,7 +1106,6 @@
           <t>TESLA-718</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1145,7 +1135,6 @@
           <t>TESLA-719</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1220,12 +1209,11 @@
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E24" t="n">
         <v>4</v>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1233,7 +1221,7 @@
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>No catalogue photo yet.</t>
+          <t>No catalogue photo yet. Rate 24 Oct 2026: ₹81 → ₹78.</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1231,6 @@
           <t>TESLA-722</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1273,7 +1260,6 @@
           <t>TESLA-751</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1303,7 +1289,6 @@
           <t>TESLA-752</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1333,7 +1318,6 @@
           <t>TESLA-753</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Clutchers</t>
@@ -1401,7 +1385,6 @@
           <t>100 PC NYLON RUBBER</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1413,7 +1396,6 @@
       <c r="E30" t="n">
         <v>1</v>
       </c>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1438,7 +1420,7 @@
         </is>
       </c>
       <c r="D31" s="5" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>1</v>
@@ -1455,7 +1437,7 @@
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Not the same as RC-300 fur chimta (clutchers, ₹90).</t>
+          <t>Not the same as RC-300 fur chimta (clutchers, ₹90). Rate 24 Oct 2026: ₹57 → ₹60.</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1447,6 @@
           <t>322</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1495,14 +1476,13 @@
           <t>335</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>36</v>
+        <v>37.5</v>
       </c>
       <c r="E33" t="n">
         <v>6</v>
@@ -1517,7 +1497,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹36 → ₹37.5.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1525,7 +1509,6 @@
           <t>349</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1555,7 +1538,6 @@
           <t>355</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1585,7 +1567,6 @@
           <t>36 PC NYLON RUBBER</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1622,7 +1603,7 @@
         </is>
       </c>
       <c r="D37" s="5" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>8</v>
@@ -1639,7 +1620,7 @@
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Not the same as RC-400 fur chimta (clutchers, ₹150).</t>
+          <t>Not the same as RC-400 fur chimta (clutchers, ₹150). Rate 24 Oct 2026: ₹63 → ₹66.</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1630,6 @@
           <t>430</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1661,7 +1641,6 @@
       <c r="E38" t="n">
         <v>4</v>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1679,7 +1658,6 @@
           <t>432</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1709,7 +1687,6 @@
           <t>433</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1739,7 +1716,6 @@
           <t>434</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1769,7 +1745,6 @@
           <t>437</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1781,7 +1756,6 @@
       <c r="E42" t="n">
         <v>4</v>
       </c>
-      <c r="F42" t="inlineStr"/>
       <c r="G42" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1799,7 +1773,6 @@
           <t>438</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1859,7 +1832,6 @@
           <t>903</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1889,7 +1861,6 @@
           <t>912</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1901,7 +1872,6 @@
       <c r="E46" t="n">
         <v>5</v>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1919,7 +1889,6 @@
           <t>913</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1931,7 +1900,6 @@
       <c r="E47" t="n">
         <v>5</v>
       </c>
-      <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1949,7 +1917,6 @@
           <t>914</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1961,7 +1928,6 @@
       <c r="E48" t="n">
         <v>6</v>
       </c>
-      <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
         <is>
           <t>Y</t>
@@ -1979,7 +1945,6 @@
           <t>917</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -1991,7 +1956,6 @@
       <c r="E49" t="n">
         <v>5</v>
       </c>
-      <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2009,7 +1973,6 @@
           <t>920</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2039,7 +2002,6 @@
           <t>931</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2069,7 +2031,6 @@
           <t>933</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2081,7 +2042,6 @@
       <c r="E52" t="n">
         <v>6</v>
       </c>
-      <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2099,7 +2059,6 @@
           <t>934</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2129,7 +2088,6 @@
           <t>940</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2159,7 +2117,6 @@
           <t>941</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2171,7 +2128,6 @@
       <c r="E55" t="n">
         <v>5</v>
       </c>
-      <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2189,7 +2145,6 @@
           <t>945</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2201,7 +2156,6 @@
       <c r="E56" t="n">
         <v>6</v>
       </c>
-      <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2219,7 +2173,6 @@
           <t>952</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2249,7 +2202,6 @@
           <t>960</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2279,14 +2231,13 @@
           <t>965</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D59" s="2" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E59" t="n">
         <v>10</v>
@@ -2301,7 +2252,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H59" s="3" t="inlineStr"/>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹39 → ₹42.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2309,7 +2264,6 @@
           <t>967</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2339,7 +2293,6 @@
           <t>980</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2369,7 +2322,6 @@
           <t>986</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2399,7 +2351,6 @@
           <t>991</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2429,14 +2380,13 @@
           <t>993</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D64" s="2" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E64" t="n">
         <v>5</v>
@@ -2451,7 +2401,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H64" s="3" t="inlineStr"/>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹57 → ₹60.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2459,14 +2413,13 @@
           <t>996</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D65" s="2" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="E65" t="n">
         <v>5</v>
@@ -2481,7 +2434,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹54 → ₹57.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2489,14 +2446,13 @@
           <t>998</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D66" s="2" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E66" t="n">
         <v>5</v>
@@ -2511,7 +2467,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H66" s="3" t="inlineStr"/>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹60 → ₹63.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2519,14 +2479,13 @@
           <t>BS-01</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D67" s="2" t="n">
-        <v>58.5</v>
+        <v>57</v>
       </c>
       <c r="E67" t="n">
         <v>6</v>
@@ -2541,7 +2500,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H67" s="3" t="inlineStr"/>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹58.5 → ₹57.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2549,7 +2512,6 @@
           <t>BS-02</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2579,14 +2541,13 @@
           <t>BS-03</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D69" s="2" t="n">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="E69" t="n">
         <v>3</v>
@@ -2601,7 +2562,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H69" s="3" t="inlineStr"/>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹114 → ₹105.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2609,19 +2574,17 @@
           <t>D-01</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D70" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E70" t="n">
         <v>12</v>
       </c>
-      <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2629,7 +2592,7 @@
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
-          <t>No catalogue photo yet.</t>
+          <t>No catalogue photo yet. Rate 24 Oct 2026: ₹16 → ₹17.</t>
         </is>
       </c>
     </row>
@@ -2639,14 +2602,13 @@
           <t>D-02</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D71" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E71" t="n">
         <v>12</v>
@@ -2661,7 +2623,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H71" s="3" t="inlineStr"/>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹16 → ₹17.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2669,7 +2635,6 @@
           <t>D-03</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2699,14 +2664,13 @@
           <t>D-04</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D73" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E73" t="n">
         <v>12</v>
@@ -2721,7 +2685,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H73" s="3" t="inlineStr"/>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹16 → ₹17.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2729,7 +2697,6 @@
           <t>D-05</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2759,14 +2726,13 @@
           <t>D-06</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D75" s="2" t="n">
-        <v>13.5</v>
+        <v>14</v>
       </c>
       <c r="E75" t="n">
         <v>12</v>
@@ -2781,7 +2747,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H75" s="3" t="inlineStr"/>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹13.5 → ₹14.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2789,7 +2759,6 @@
           <t>D-07</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2819,14 +2788,13 @@
           <t>D-08</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D77" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E77" t="n">
         <v>12</v>
@@ -2841,7 +2809,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H77" s="3" t="inlineStr"/>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹12 → ₹13.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2849,7 +2821,6 @@
           <t>D-09</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -2861,7 +2832,6 @@
       <c r="E78" t="n">
         <v>12</v>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>Y</t>
@@ -2879,14 +2849,13 @@
           <t>D-10</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D79" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E79" t="n">
         <v>12</v>
@@ -2901,7 +2870,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H79" s="3" t="inlineStr"/>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹16 → ₹17.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
@@ -3011,7 +2984,6 @@
           <t>MOBILON CARD</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3023,7 +2995,6 @@
       <c r="E83" t="n">
         <v>12</v>
       </c>
-      <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3041,7 +3012,6 @@
           <t>PS-01</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3053,7 +3023,6 @@
       <c r="E84" t="n">
         <v>6</v>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3105,7 +3074,6 @@
           <t>RC-202</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3135,7 +3103,6 @@
           <t>RC-254</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3147,7 +3114,6 @@
       <c r="E87" t="n">
         <v>3</v>
       </c>
-      <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3176,7 +3142,7 @@
         </is>
       </c>
       <c r="D88" s="2" t="n">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E88" t="n">
         <v>6</v>
@@ -3191,7 +3157,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H88" s="3" t="inlineStr"/>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹81 → ₹84.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3215,7 +3185,6 @@
       <c r="E89" t="n">
         <v>10</v>
       </c>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3233,7 +3202,6 @@
           <t>RC-611</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3245,7 +3213,6 @@
       <c r="E90" t="n">
         <v>6</v>
       </c>
-      <c r="F90" t="inlineStr"/>
       <c r="G90" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3263,7 +3230,6 @@
           <t>RC-612</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3275,7 +3241,6 @@
       <c r="E91" t="n">
         <v>6</v>
       </c>
-      <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3304,7 +3269,7 @@
         </is>
       </c>
       <c r="D92" s="5" t="n">
-        <v>30</v>
+        <v>31.5</v>
       </c>
       <c r="E92" s="4" t="n">
         <v>10</v>
@@ -3321,7 +3286,7 @@
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>Catalogue says T-613 – same item?</t>
+          <t>Catalogue says T-613 – same item? Rate 24 Oct 2026: ₹30 → ₹31.5.</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3303,7 @@
         </is>
       </c>
       <c r="D93" s="5" t="n">
-        <v>30</v>
+        <v>31.5</v>
       </c>
       <c r="E93" s="4" t="n">
         <v>10</v>
@@ -3355,7 +3320,7 @@
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>Catalogue says T-614 – same item?</t>
+          <t>Catalogue says T-614 – same item? Rate 24 Oct 2026: ₹30 → ₹31.5.</t>
         </is>
       </c>
     </row>
@@ -3365,19 +3330,17 @@
           <t>RC-615</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D94" s="2" t="n">
-        <v>30</v>
+        <v>31.5</v>
       </c>
       <c r="E94" t="n">
         <v>10</v>
       </c>
-      <c r="F94" t="inlineStr"/>
       <c r="G94" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3385,7 +3348,7 @@
       </c>
       <c r="H94" s="3" t="inlineStr">
         <is>
-          <t>No catalogue photo yet.</t>
+          <t>No catalogue photo yet. Rate 24 Oct 2026: ₹30 → ₹31.5.</t>
         </is>
       </c>
     </row>
@@ -3395,7 +3358,6 @@
           <t>RC-616</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3407,7 +3369,6 @@
       <c r="E95" t="n">
         <v>10</v>
       </c>
-      <c r="F95" t="inlineStr"/>
       <c r="G95" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3425,7 +3386,6 @@
           <t>RC-617</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -3523,14 +3483,13 @@
           <t>RJ-1001</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E99" t="n">
         <v>5</v>
@@ -3545,7 +3504,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H99" s="3" t="inlineStr"/>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹90 → ₹96.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3553,14 +3516,13 @@
           <t>RJ-1002</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="E100" t="n">
         <v>6</v>
@@ -3575,7 +3537,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H100" s="3" t="inlineStr"/>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹90 → ₹102.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3583,14 +3549,13 @@
           <t>RJ-1003</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="E101" t="n">
         <v>6</v>
@@ -3605,7 +3570,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H101" s="3" t="inlineStr"/>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹96 → ₹108.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3613,14 +3582,13 @@
           <t>RJ-1004</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E102" t="n">
         <v>6</v>
@@ -3635,7 +3603,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H102" s="3" t="inlineStr"/>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹51 → ₹54.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3643,19 +3615,17 @@
           <t>RJ-1005</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>108</v>
+        <v>120</v>
       </c>
       <c r="E103" t="n">
         <v>6</v>
       </c>
-      <c r="F103" t="inlineStr"/>
       <c r="G103" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3663,7 +3633,7 @@
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>No catalogue photo yet.</t>
+          <t>No catalogue photo yet. Rate 24 Oct 2026: ₹108 → ₹120.</t>
         </is>
       </c>
     </row>
@@ -3673,19 +3643,17 @@
           <t>RJ-1006</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E104" t="n">
         <v>6</v>
       </c>
-      <c r="F104" t="inlineStr"/>
       <c r="G104" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3693,7 +3661,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>No catalogue photo yet.</t>
+          <t>No catalogue photo yet. Rate 24 Oct 2026: ₹72 → ₹78.</t>
         </is>
       </c>
     </row>
@@ -3703,19 +3671,17 @@
           <t>RJ-1007</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="E105" t="n">
         <v>3</v>
       </c>
-      <c r="F105" t="inlineStr"/>
       <c r="G105" t="inlineStr">
         <is>
           <t>Y</t>
@@ -3723,7 +3689,7 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>No catalogue photo yet.</t>
+          <t>No catalogue photo yet. Rate 24 Oct 2026: ₹102 → ₹108.</t>
         </is>
       </c>
     </row>
@@ -3744,7 +3710,7 @@
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="E106" t="n">
         <v>10</v>
@@ -3759,7 +3725,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H106" s="3" t="inlineStr"/>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹81 → ₹78.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -3812,7 +3782,7 @@
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E108" t="n">
         <v>10</v>
@@ -3827,7 +3797,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H108" s="3" t="inlineStr"/>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹90 → ₹87.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -3846,7 +3820,7 @@
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="E109" t="n">
         <v>10</v>
@@ -3861,7 +3835,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H109" s="3" t="inlineStr"/>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹108 → ₹105.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -3880,7 +3858,7 @@
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="E110" t="n">
         <v>10</v>
@@ -3895,7 +3873,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H110" s="3" t="inlineStr"/>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹126 → ₹120.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -3914,7 +3896,7 @@
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>150</v>
+        <v>138</v>
       </c>
       <c r="E111" t="n">
         <v>10</v>
@@ -3929,7 +3911,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H111" s="3" t="inlineStr"/>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹150 → ₹138.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -3948,7 +3934,7 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>180</v>
+        <v>156</v>
       </c>
       <c r="E112" t="n">
         <v>10</v>
@@ -3963,7 +3949,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H112" s="3" t="inlineStr"/>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹180 → ₹156.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -4025,7 +4015,6 @@
       <c r="E114" t="n">
         <v>6</v>
       </c>
-      <c r="F114" t="inlineStr"/>
       <c r="G114" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4054,7 +4043,7 @@
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="E115" t="n">
         <v>10</v>
@@ -4069,7 +4058,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H115" s="3" t="inlineStr"/>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹198 → ₹180.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4088,7 +4081,7 @@
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>220</v>
+        <v>204</v>
       </c>
       <c r="E116" t="n">
         <v>10</v>
@@ -4103,7 +4096,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H116" s="3" t="inlineStr"/>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹220 → ₹204.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4111,7 +4108,6 @@
           <t>SUMO-RINKLE</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -4141,7 +4137,6 @@
           <t>TIER RUBED</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -4153,7 +4148,6 @@
       <c r="E118" t="n">
         <v>10</v>
       </c>
-      <c r="F118" t="inlineStr"/>
       <c r="G118" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4171,7 +4165,6 @@
           <t>XL 30 PC</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -4231,7 +4224,6 @@
           <t>XL 72 PC RUBED</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
           <t>Scrunchies</t>
@@ -4243,7 +4235,6 @@
       <c r="E121" t="n">
         <v>6</v>
       </c>
-      <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4261,14 +4252,13 @@
           <t>XXL 30 PC</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
       <c r="C122" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D122" s="2" t="n">
-        <v>28.5</v>
+        <v>30</v>
       </c>
       <c r="E122" t="n">
         <v>10</v>
@@ -4283,7 +4273,11 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="H122" s="3" t="inlineStr"/>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>Rate 24 Oct 2026: ₹28.5 → ₹30.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4291,19 +4285,17 @@
           <t>XXL 72 PC RUBED</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
           <t>Scrunchies</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="E123" t="n">
         <v>6</v>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>Y</t>
@@ -4311,7 +4303,7 @@
       </c>
       <c r="H123" s="3" t="inlineStr">
         <is>
-          <t>No catalogue photo yet.</t>
+          <t>No catalogue photo yet. Rate 24 Oct 2026: ₹60 → ₹63.</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4313,6 @@
           <t>278</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4351,7 +4342,6 @@
           <t>503</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4415,7 +4405,6 @@
           <t>RC-253</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4445,7 +4434,6 @@
           <t>RC-255</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4475,7 +4463,6 @@
           <t>RC-256</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4505,7 +4492,6 @@
           <t>RC-258</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4535,7 +4521,6 @@
           <t>RC-259</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4565,7 +4550,6 @@
           <t>RC-264</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4595,7 +4579,6 @@
           <t>RC-265</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4625,7 +4608,6 @@
           <t>RC-266</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4655,7 +4637,6 @@
           <t>RC-267</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4685,7 +4666,6 @@
           <t>RC-274</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4715,7 +4695,6 @@
           <t>RC-275</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
           <t>Tie Bow</t>
@@ -4834,162 +4813,6 @@
       <c r="H140" s="6" t="inlineStr">
         <is>
           <t>Carton charge, not a product. Keep hidden (or tell us if it should be added to orders).</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="7" t="inlineStr"/>
-      <c r="B141" s="7" t="inlineStr"/>
-      <c r="C141" s="7" t="inlineStr">
-        <is>
-          <t>Clutchers</t>
-        </is>
-      </c>
-      <c r="D141" s="8" t="n"/>
-      <c r="E141" s="7" t="n"/>
-      <c r="F141" s="7" t="inlineStr">
-        <is>
-          <t>RC 200</t>
-        </is>
-      </c>
-      <c r="G141" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H141" s="9" t="inlineStr">
-        <is>
-          <t>Catalogue item with NO rate – fill in Code, Rate and Packet, or leave empty for 'price on request'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="7" t="inlineStr"/>
-      <c r="B142" s="7" t="inlineStr"/>
-      <c r="C142" s="7" t="inlineStr">
-        <is>
-          <t>Scrunchies</t>
-        </is>
-      </c>
-      <c r="D142" s="8" t="n"/>
-      <c r="E142" s="7" t="n"/>
-      <c r="F142" s="7" t="inlineStr">
-        <is>
-          <t>968</t>
-        </is>
-      </c>
-      <c r="G142" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H142" s="9" t="inlineStr">
-        <is>
-          <t>Catalogue item with NO rate – fill in Code, Rate and Packet, or leave empty for 'price on request'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="7" t="inlineStr"/>
-      <c r="B143" s="7" t="inlineStr"/>
-      <c r="C143" s="7" t="inlineStr">
-        <is>
-          <t>Scrunchies</t>
-        </is>
-      </c>
-      <c r="D143" s="8" t="n"/>
-      <c r="E143" s="7" t="n"/>
-      <c r="F143" s="7" t="inlineStr">
-        <is>
-          <t>959</t>
-        </is>
-      </c>
-      <c r="G143" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H143" s="9" t="inlineStr">
-        <is>
-          <t>Catalogue item with NO rate – fill in Code, Rate and Packet, or leave empty for 'price on request'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="7" t="inlineStr"/>
-      <c r="B144" s="7" t="inlineStr"/>
-      <c r="C144" s="7" t="inlineStr">
-        <is>
-          <t>Tie Bow</t>
-        </is>
-      </c>
-      <c r="D144" s="8" t="n"/>
-      <c r="E144" s="7" t="n"/>
-      <c r="F144" s="7" t="inlineStr">
-        <is>
-          <t>RC 307</t>
-        </is>
-      </c>
-      <c r="G144" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H144" s="9" t="inlineStr">
-        <is>
-          <t>Catalogue item with NO rate – fill in Code, Rate and Packet, or leave empty for 'price on request'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="7" t="inlineStr"/>
-      <c r="B145" s="7" t="inlineStr"/>
-      <c r="C145" s="7" t="inlineStr">
-        <is>
-          <t>Tie Bow</t>
-        </is>
-      </c>
-      <c r="D145" s="8" t="n"/>
-      <c r="E145" s="7" t="n"/>
-      <c r="F145" s="7" t="inlineStr">
-        <is>
-          <t>RC 271</t>
-        </is>
-      </c>
-      <c r="G145" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H145" s="9" t="inlineStr">
-        <is>
-          <t>Catalogue item with NO rate – fill in Code, Rate and Packet, or leave empty for 'price on request'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="7" t="inlineStr"/>
-      <c r="B146" s="7" t="inlineStr"/>
-      <c r="C146" s="7" t="inlineStr">
-        <is>
-          <t>Tie Bow</t>
-        </is>
-      </c>
-      <c r="D146" s="8" t="n"/>
-      <c r="E146" s="7" t="n"/>
-      <c r="F146" s="7" t="inlineStr">
-        <is>
-          <t>RC 262</t>
-        </is>
-      </c>
-      <c r="G146" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H146" s="9" t="inlineStr">
-        <is>
-          <t>Catalogue item with NO rate – fill in Code, Rate and Packet, or leave empty for 'price on request'.</t>
         </is>
       </c>
     </row>
@@ -5017,9 +4840,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -5076,9 +4897,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Website: rates for 8 photo items that were "Price on request"
TESLA-710 126/1, 986 86/6, 991 104/4, 36 PC NYLON RUBBER 26/6, 1126 92/4,
RC-253 140/3, RC-511 96/4, RC-265 150/3 (rate per dozen / dozen per packet,
as given by Raj). 1127 still has no rate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XttcUphWVwshiXCPpeS9yb
</commit_message>
<xml_diff>
--- a/website/Website Rates (for Google Sheet).xlsx
+++ b/website/Website Rates (for Google Sheet).xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H116"/>
+  <dimension ref="A1:H124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4348,26 +4348,285 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CARTOON</t>
+          <t>TESLA-710</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Clutchers</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>403</v>
+        <v>126</v>
       </c>
       <c r="E116" t="n">
         <v>1</v>
       </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>TESLA 710</t>
+        </is>
+      </c>
       <c r="G116" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>986</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Scrunchies</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>86</v>
+      </c>
+      <c r="E117" t="n">
+        <v>6</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>986</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>991</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Scrunchies</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>104</v>
+      </c>
+      <c r="E118" t="n">
+        <v>4</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>991</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>36 PC NYLON RUBBER</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Scrunchies</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>26</v>
+      </c>
+      <c r="E119" t="n">
+        <v>6</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>36 PC NYLON RUBBER</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1126</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Scrunchies</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>92</v>
+      </c>
+      <c r="E120" t="n">
+        <v>4</v>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>RC-253</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Tie Bow</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>140</v>
+      </c>
+      <c r="E121" t="n">
+        <v>3</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>RC 253</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>RC-511</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Tie Bow</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>96</v>
+      </c>
+      <c r="E122" t="n">
+        <v>4</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>RC 511</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>RC-265</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Tie Bow</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>150</v>
+      </c>
+      <c r="E123" t="n">
+        <v>3</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>RC 265</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Rate given by Raj, 29 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>CARTOON</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>403</v>
+      </c>
+      <c r="E124" t="n">
+        <v>1</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr">
+      <c r="H124" t="inlineStr">
         <is>
           <t>Carton charge, not a product. Keep hidden.</t>
         </is>

</xml_diff>